<commit_message>
import and config tab
</commit_message>
<xml_diff>
--- a/Produkty/BULL S.xlsx
+++ b/Produkty/BULL S.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Oskar\Desktop\MT-GO-WEB\Produkty\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{834CC361-D3B6-4848-B553-CB2FF5717EAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25244084-9B78-47A1-8227-7FC81C0FA5EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -676,7 +676,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q34"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
   <cols>
     <col min="1" max="1" width="12.8125" customWidth="1"/>
     <col min="2" max="2" width="25.6875" customWidth="1"/>
@@ -687,7 +687,7 @@
     <col min="11" max="11" width="12.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.5">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -740,7 +740,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:17" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.5">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -793,7 +793,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:17" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.5">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -846,7 +846,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:17" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.5">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -899,7 +899,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:17" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.5">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -952,7 +952,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:17" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.5">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -1005,7 +1005,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:17" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.5">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -1058,7 +1058,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:17" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.5">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -1111,7 +1111,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:17" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.5">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -1164,7 +1164,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:17" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.5">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -1217,7 +1217,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:17" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.5">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -1270,7 +1270,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:17" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.5">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -1323,7 +1323,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:17" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.5">
       <c r="A13" t="s">
         <v>16</v>
       </c>
@@ -1376,7 +1376,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:17" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.5">
       <c r="A14" t="s">
         <v>16</v>
       </c>
@@ -1429,7 +1429,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:17" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.5">
       <c r="A15" t="s">
         <v>16</v>
       </c>
@@ -1482,7 +1482,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="16" spans="1:17" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.5">
       <c r="A16" t="s">
         <v>16</v>
       </c>
@@ -1535,7 +1535,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="1:17" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="17" spans="1:17" x14ac:dyDescent="0.5">
       <c r="A17" t="s">
         <v>16</v>
       </c>
@@ -1588,7 +1588,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="18" spans="1:17" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="18" spans="1:17" x14ac:dyDescent="0.5">
       <c r="A18" t="s">
         <v>16</v>
       </c>
@@ -1641,7 +1641,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="19" spans="1:17" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="19" spans="1:17" x14ac:dyDescent="0.5">
       <c r="A19" t="s">
         <v>16</v>
       </c>
@@ -1694,7 +1694,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="20" spans="1:17" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="20" spans="1:17" x14ac:dyDescent="0.5">
       <c r="A20" t="s">
         <v>16</v>
       </c>
@@ -1747,7 +1747,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:17" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="21" spans="1:17" x14ac:dyDescent="0.5">
       <c r="A21" t="s">
         <v>16</v>
       </c>
@@ -1800,7 +1800,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="1:17" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="22" spans="1:17" x14ac:dyDescent="0.5">
       <c r="A22" t="s">
         <v>16</v>
       </c>
@@ -1853,7 +1853,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="23" spans="1:17" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="23" spans="1:17" x14ac:dyDescent="0.5">
       <c r="A23" t="s">
         <v>16</v>
       </c>
@@ -1906,7 +1906,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="24" spans="1:17" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="24" spans="1:17" x14ac:dyDescent="0.5">
       <c r="A24" t="s">
         <v>16</v>
       </c>
@@ -1959,7 +1959,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="25" spans="1:17" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="25" spans="1:17" x14ac:dyDescent="0.5">
       <c r="A25" t="s">
         <v>16</v>
       </c>
@@ -2012,7 +2012,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="26" spans="1:17" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="26" spans="1:17" x14ac:dyDescent="0.5">
       <c r="A26" t="s">
         <v>16</v>
       </c>
@@ -2065,7 +2065,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:17" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="27" spans="1:17" x14ac:dyDescent="0.5">
       <c r="A27" t="s">
         <v>16</v>
       </c>
@@ -2118,7 +2118,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="28" spans="1:17" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="28" spans="1:17" x14ac:dyDescent="0.5">
       <c r="A28" t="s">
         <v>16</v>
       </c>
@@ -2171,7 +2171,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="29" spans="1:17" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="29" spans="1:17" x14ac:dyDescent="0.5">
       <c r="A29" t="s">
         <v>16</v>
       </c>
@@ -2224,7 +2224,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="30" spans="1:17" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="30" spans="1:17" x14ac:dyDescent="0.5">
       <c r="A30" t="s">
         <v>16</v>
       </c>
@@ -2277,7 +2277,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="31" spans="1:17" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="31" spans="1:17" x14ac:dyDescent="0.5">
       <c r="A31" t="s">
         <v>16</v>
       </c>
@@ -2330,7 +2330,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="32" spans="1:17" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="32" spans="1:17" x14ac:dyDescent="0.5">
       <c r="A32" t="s">
         <v>16</v>
       </c>
@@ -2383,7 +2383,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="33" spans="1:17" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="33" spans="1:17" x14ac:dyDescent="0.5">
       <c r="A33" t="s">
         <v>16</v>
       </c>
@@ -2436,7 +2436,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="34" spans="1:17" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="34" spans="1:17" x14ac:dyDescent="0.5">
       <c r="A34" t="s">
         <v>16</v>
       </c>
@@ -2492,7 +2492,7 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:Q34" numberStoredAsText="1"/>
+    <ignoredError sqref="A2:Q34 A1:B1 D1:Q1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>